<commit_message>
Added paired t-test and changed internal data retrieval
</commit_message>
<xml_diff>
--- a/examples/Olink_Finished_Example/delivery/data/Data_With_Analysis.xlsx
+++ b/examples/Olink_Finished_Example/delivery/data/Data_With_Analysis.xlsx
@@ -12587,7 +12587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12598,6 +12598,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12641,6 +12642,11 @@
           <t>Sample 7</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t># Missing</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -12659,6 +12665,9 @@
         <v>0.1893143655000005</v>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="3" t="n">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>